<commit_message>
All the changes are made after testing - add filter on admin dashboard, delete user panel from admin side, gmail should be starts with alphabets, hours or day wise booking
</commit_message>
<xml_diff>
--- a/Table Data.xlsx
+++ b/Table Data.xlsx
@@ -4,19 +4,19 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="108" windowWidth="22980" windowHeight="9288"/>
+    <workbookView xWindow="0" yWindow="108" windowWidth="22980" windowHeight="9288" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Tables" sheetId="1" r:id="rId1"/>
+    <sheet name="Gantt Chart" sheetId="2" r:id="rId2"/>
+    <sheet name="Modify to be done" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="160">
   <si>
     <t xml:space="preserve">User Table </t>
   </si>
@@ -415,6 +415,87 @@
   </si>
   <si>
     <t>vehicle_count</t>
+  </si>
+  <si>
+    <t>Phases</t>
+  </si>
+  <si>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>Development</t>
+  </si>
+  <si>
+    <t>Testing</t>
+  </si>
+  <si>
+    <t>Problem Statement with proposed solution</t>
+  </si>
+  <si>
+    <t>Tasks</t>
+  </si>
+  <si>
+    <t>DFD, Database schema, wireframes &amp; test cases</t>
+  </si>
+  <si>
+    <t>Check Test case</t>
+  </si>
+  <si>
+    <t>GoHigh Rentals</t>
+  </si>
+  <si>
+    <t>Coding phase-Pages of Website</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S. No. </t>
+  </si>
+  <si>
+    <t>Change to be done</t>
+  </si>
+  <si>
+    <t>Add filter on stats card</t>
+  </si>
+  <si>
+    <t>Add profile button on dashboard (in which user can see their previous bookings and user have an option for update their profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Many booking from same user it should not be done (generate a error message you are not able to book many bookings for same date for same time) </t>
+  </si>
+  <si>
+    <t>Add invoice next to action of completed trips</t>
+  </si>
+  <si>
+    <t>Add option of user review add file extensions like images, video etc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add admin </t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>In dashboard, check availability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add filter on admin dashboard in bookings where dates, vehicles, accept, cancel, confirmed , complete bookings can be filter out </t>
+  </si>
+  <si>
+    <t>Admin can be delete user from their panel</t>
+  </si>
+  <si>
+    <t>Gmail should be alphanumeric like phone@gmai.. Is not allowed  startswith alphabets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking should be hour or day wise have to modify the pricing table </t>
+  </si>
+  <si>
+    <t>Correct the price in destination like it show 2500 per day but when user click on book now the bill is created of 330</t>
+  </si>
+  <si>
+    <t>When user cancel the booking admin don’t have option for cancel or accept that booking and notify to admin that user cancelled this booking same as for user</t>
   </si>
 </sst>
 </file>
@@ -424,7 +505,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -432,8 +513,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -452,8 +541,50 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF3C7F8C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -633,11 +764,103 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -693,6 +916,38 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -711,12 +966,34 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF3C7F8C"/>
+    </mruColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1005,6 +1282,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FFFFC000"/>
+  </sheetPr>
   <dimension ref="A1:O39"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
@@ -1026,21 +1306,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="I1" s="28" t="s">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="I1" s="46" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="29"/>
-      <c r="K1" s="29"/>
-      <c r="L1" s="29"/>
-      <c r="M1" s="30"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="48"/>
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="10" t="s">
@@ -1429,23 +1709,23 @@
     </row>
     <row r="14" spans="1:14" ht="15" thickBot="1"/>
     <row r="15" spans="1:14">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="43" t="s">
         <v>69</v>
       </c>
-      <c r="B15" s="26"/>
-      <c r="C15" s="26"/>
-      <c r="D15" s="27"/>
-      <c r="F15" s="25" t="s">
+      <c r="B15" s="44"/>
+      <c r="C15" s="44"/>
+      <c r="D15" s="45"/>
+      <c r="F15" s="43" t="s">
         <v>76</v>
       </c>
-      <c r="G15" s="26"/>
-      <c r="H15" s="26"/>
-      <c r="I15" s="26"/>
-      <c r="J15" s="26"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="25"/>
-      <c r="N15" s="26"/>
+      <c r="G15" s="44"/>
+      <c r="H15" s="44"/>
+      <c r="I15" s="44"/>
+      <c r="J15" s="44"/>
+      <c r="K15" s="44"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="43"/>
+      <c r="N15" s="44"/>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="5" t="s">
@@ -1900,24 +2180,24 @@
     </row>
     <row r="27" spans="1:15" ht="15" thickBot="1"/>
     <row r="28" spans="1:15">
-      <c r="A28" s="25" t="s">
+      <c r="A28" s="43" t="s">
         <v>115</v>
       </c>
-      <c r="B28" s="26"/>
-      <c r="C28" s="26"/>
-      <c r="D28" s="26"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
-      <c r="G28" s="27"/>
-      <c r="I28" s="25" t="s">
+      <c r="B28" s="44"/>
+      <c r="C28" s="44"/>
+      <c r="D28" s="44"/>
+      <c r="E28" s="44"/>
+      <c r="F28" s="44"/>
+      <c r="G28" s="45"/>
+      <c r="I28" s="43" t="s">
         <v>124</v>
       </c>
-      <c r="J28" s="26"/>
-      <c r="K28" s="26"/>
-      <c r="L28" s="26"/>
-      <c r="M28" s="26"/>
-      <c r="N28" s="26"/>
-      <c r="O28" s="27"/>
+      <c r="J28" s="44"/>
+      <c r="K28" s="44"/>
+      <c r="L28" s="44"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="44"/>
+      <c r="O28" s="45"/>
     </row>
     <row r="29" spans="1:15">
       <c r="A29" s="5" t="s">
@@ -2420,18 +2700,294 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="46.6640625" customWidth="1"/>
+    <col min="2" max="2" width="20.109375" customWidth="1"/>
+    <col min="3" max="6" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="50" t="s">
+        <v>142</v>
+      </c>
+      <c r="B1" s="51"/>
+    </row>
+    <row r="2" spans="1:9" ht="15" thickBot="1">
+      <c r="A2" s="52"/>
+      <c r="B2" s="53"/>
+    </row>
+    <row r="3" spans="1:9" ht="15" thickBot="1"/>
+    <row r="4" spans="1:9">
+      <c r="A4" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" s="31">
+        <v>46050</v>
+      </c>
+      <c r="D4" s="31">
+        <v>46051</v>
+      </c>
+      <c r="E4" s="31">
+        <v>46052</v>
+      </c>
+      <c r="F4" s="31">
+        <v>46073</v>
+      </c>
+      <c r="G4" s="31">
+        <v>46094</v>
+      </c>
+      <c r="H4" s="31">
+        <v>46095</v>
+      </c>
+      <c r="I4" s="31">
+        <v>46096</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>134</v>
+      </c>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="C6" s="32"/>
+      <c r="D6" s="34"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" s="29" t="s">
+        <v>136</v>
+      </c>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+    </row>
+    <row r="8" spans="1:9" ht="15" thickBot="1">
+      <c r="A8" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>137</v>
+      </c>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="36"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A1:B2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <sheetPr>
+    <tabColor rgb="FF00B0F0"/>
+  </sheetPr>
+  <dimension ref="B3:E17"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="125.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5">
+      <c r="B3" s="40"/>
+      <c r="C3" s="42" t="s">
+        <v>144</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>145</v>
+      </c>
+      <c r="E3" s="42"/>
+    </row>
+    <row r="4" spans="2:5">
+      <c r="B4" s="40"/>
+      <c r="C4" s="41">
+        <v>1</v>
+      </c>
+      <c r="D4" s="40" t="s">
+        <v>146</v>
+      </c>
+      <c r="E4" s="40"/>
+    </row>
+    <row r="5" spans="2:5">
+      <c r="B5" s="40"/>
+      <c r="C5" s="41">
+        <v>2</v>
+      </c>
+      <c r="D5" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="E5" s="40" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5">
+      <c r="B6" s="40"/>
+      <c r="C6" s="41">
+        <v>3</v>
+      </c>
+      <c r="D6" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="E6" s="40" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
+      <c r="B7" s="40"/>
+      <c r="C7" s="41">
+        <v>4</v>
+      </c>
+      <c r="D7" s="40" t="s">
+        <v>149</v>
+      </c>
+      <c r="E7" s="40" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
+      <c r="B8" s="40"/>
+      <c r="C8" s="41">
+        <v>5</v>
+      </c>
+      <c r="D8" s="40" t="s">
+        <v>150</v>
+      </c>
+      <c r="E8" s="40" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5">
+      <c r="B9" s="40"/>
+      <c r="C9" s="41">
+        <v>6</v>
+      </c>
+      <c r="D9" s="40" t="s">
+        <v>153</v>
+      </c>
+      <c r="E9" s="40" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5">
+      <c r="B10" s="40"/>
+      <c r="C10" s="41">
+        <v>7</v>
+      </c>
+      <c r="D10" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="E10" s="40"/>
+    </row>
+    <row r="11" spans="2:5">
+      <c r="B11" s="54">
+        <v>46098</v>
+      </c>
+      <c r="C11" s="41">
+        <v>8</v>
+      </c>
+      <c r="D11" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" s="40"/>
+    </row>
+    <row r="12" spans="2:5">
+      <c r="B12" s="40"/>
+      <c r="C12" s="41">
+        <v>9</v>
+      </c>
+      <c r="D12" s="40" t="s">
+        <v>155</v>
+      </c>
+      <c r="E12" s="40"/>
+    </row>
+    <row r="13" spans="2:5">
+      <c r="B13" s="40"/>
+      <c r="C13" s="41">
+        <v>10</v>
+      </c>
+      <c r="D13" s="40" t="s">
+        <v>156</v>
+      </c>
+      <c r="E13" s="40"/>
+    </row>
+    <row r="14" spans="2:5">
+      <c r="B14" s="40"/>
+      <c r="C14" s="41">
+        <v>11</v>
+      </c>
+      <c r="D14" s="40" t="s">
+        <v>157</v>
+      </c>
+      <c r="E14" s="40"/>
+    </row>
+    <row r="15" spans="2:5">
+      <c r="B15" s="40"/>
+      <c r="C15" s="41">
+        <v>12</v>
+      </c>
+      <c r="D15" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="E15" s="40"/>
+    </row>
+    <row r="16" spans="2:5">
+      <c r="B16" s="40"/>
+      <c r="C16" s="41">
+        <v>13</v>
+      </c>
+      <c r="D16" s="55" t="s">
+        <v>159</v>
+      </c>
+      <c r="E16" s="40"/>
+    </row>
+    <row r="17" spans="3:3">
+      <c r="C17" s="39"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>